<commit_message>
Recalculate theoretical entitlement with promotion_calculator
Fee totals still come from redemption SUM and T-2. When standard.xlsx
has activity/coupon rules, calculation_engine now calls the discount,
gift, and coupon templates to fill theoretical benefit and 一致/差异.
Converter runs without rules stay 按核销明细. Xingluqiang manjian
matches 2040/136/1995; the test coupon is 200; manzeng gift qty is 98/98.

Co-authored-by: peggyzhan1 <peggyzhan1@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/samples/kuaima-verified-standard/ec101_standard库结构与当前数据.xlsx
+++ b/docs/samples/kuaima-verified-standard/ec101_standard库结构与当前数据.xlsx
@@ -464,7 +464,7 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>mvp/ec101_standard.db</t>
+          <t>docs/samples/kuaima-verified-standard/ec101_standard.db</t>
         </is>
       </c>
     </row>
@@ -562,10 +562,8 @@
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr"/>
-      <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t>（空表）</t>
-        </is>
+      <c r="E2" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -585,10 +583,8 @@
           <t>是</t>
         </is>
       </c>
-      <c r="E3" s="1" t="inlineStr">
-        <is>
-          <t>（空表）</t>
-        </is>
+      <c r="E3" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -610,7 +606,7 @@
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>（空表）</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -633,7 +629,7 @@
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>（空表）</t>
+          <t>商品</t>
         </is>
       </c>
     </row>
@@ -656,7 +652,7 @@
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>（空表）</t>
+          <t>品牌</t>
         </is>
       </c>
     </row>
@@ -679,7 +675,7 @@
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>（空表）</t>
+          <t>可口可乐</t>
         </is>
       </c>
     </row>
@@ -865,7 +861,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1091,12 +1087,12 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>participating_orders</t>
+          <t>theoretical_activity_benefit</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
-          <t>INTEGER</t>
+          <t>NUMERIC</t>
         </is>
       </c>
       <c r="C11" s="1" t="inlineStr"/>
@@ -1106,18 +1102,18 @@
         </is>
       </c>
       <c r="E11" s="1" t="n">
-        <v>136</v>
+        <v>2040</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>released_orders</t>
+          <t>theoretical_coupon_benefit</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
-          <t>INTEGER</t>
+          <t>NUMERIC</t>
         </is>
       </c>
       <c r="C12" s="1" t="inlineStr"/>
@@ -1127,18 +1123,18 @@
         </is>
       </c>
       <c r="E12" s="1" t="n">
-        <v>133</v>
+        <v>200</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>consistent_orders</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
-          <t>TEXT</t>
+          <t>INTEGER</t>
         </is>
       </c>
       <c r="C13" s="1" t="inlineStr"/>
@@ -1147,7 +1143,70 @@
           <t>是</t>
         </is>
       </c>
-      <c r="E13" s="1" t="inlineStr">
+      <c r="E13" s="1" t="n">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>participating_orders</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="inlineStr"/>
+      <c r="D14" s="1" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="E14" s="1" t="n">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>released_orders</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="C15" s="1" t="inlineStr"/>
+      <c r="D15" s="1" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="E15" s="1" t="n">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="C16" s="1" t="inlineStr"/>
+      <c r="D16" s="1" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="E16" s="1" t="inlineStr">
         <is>
           <t>calculated</t>
         </is>
@@ -1211,10 +1270,8 @@
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr"/>
-      <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t>（空表）</t>
-        </is>
+      <c r="E2" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -1234,10 +1291,8 @@
           <t>是</t>
         </is>
       </c>
-      <c r="E3" s="1" t="inlineStr">
-        <is>
-          <t>（空表）</t>
-        </is>
+      <c r="E3" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -1259,7 +1314,7 @@
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>（空表）</t>
+          <t>KM-COUPON-AUTO-001</t>
         </is>
       </c>
     </row>
@@ -1282,7 +1337,7 @@
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>（空表）</t>
+          <t>test1</t>
         </is>
       </c>
     </row>
@@ -1301,7 +1356,7 @@
       <c r="D6" s="1" t="inlineStr"/>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>（空表）</t>
+          <t>单品优惠</t>
         </is>
       </c>
     </row>
@@ -1324,7 +1379,7 @@
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>（空表）</t>
+          <t>已结束</t>
         </is>
       </c>
     </row>
@@ -1386,10 +1441,8 @@
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr"/>
-      <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t>（空表）</t>
-        </is>
+      <c r="E2" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -1409,10 +1462,8 @@
           <t>是</t>
         </is>
       </c>
-      <c r="E3" s="1" t="inlineStr">
-        <is>
-          <t>（空表）</t>
-        </is>
+      <c r="E3" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -1434,7 +1485,7 @@
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>（空表）</t>
+          <t>auto_grant</t>
         </is>
       </c>
     </row>
@@ -1457,7 +1508,7 @@
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>（空表）</t>
+          <t>2026-09-09 16:55:00</t>
         </is>
       </c>
     </row>
@@ -1474,11 +1525,7 @@
       </c>
       <c r="C6" s="1" t="inlineStr"/>
       <c r="D6" s="1" t="inlineStr"/>
-      <c r="E6" s="1" t="inlineStr">
-        <is>
-          <t>（空表）</t>
-        </is>
-      </c>
+      <c r="E6" s="1" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -1495,7 +1542,7 @@
       <c r="D7" s="1" t="inlineStr"/>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>（空表）</t>
+          <t>2026-09-09 16:55:00</t>
         </is>
       </c>
     </row>
@@ -1516,10 +1563,8 @@
           <t>是</t>
         </is>
       </c>
-      <c r="E8" s="1" t="inlineStr">
-        <is>
-          <t>（空表）</t>
-        </is>
+      <c r="E8" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -1535,10 +1580,8 @@
       </c>
       <c r="C9" s="1" t="inlineStr"/>
       <c r="D9" s="1" t="inlineStr"/>
-      <c r="E9" s="1" t="inlineStr">
-        <is>
-          <t>（空表）</t>
-        </is>
+      <c r="E9" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1554,10 +1597,8 @@
       </c>
       <c r="C10" s="1" t="inlineStr"/>
       <c r="D10" s="1" t="inlineStr"/>
-      <c r="E10" s="1" t="inlineStr">
-        <is>
-          <t>（空表）</t>
-        </is>
+      <c r="E10" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -1579,7 +1620,7 @@
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>（空表）</t>
+          <t>已结束</t>
         </is>
       </c>
     </row>
@@ -1918,10 +1959,8 @@
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr"/>
-      <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t>（空表）</t>
-        </is>
+      <c r="E2" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -1941,10 +1980,8 @@
           <t>是</t>
         </is>
       </c>
-      <c r="E3" s="1" t="inlineStr">
-        <is>
-          <t>（空表）</t>
-        </is>
+      <c r="E3" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -1966,7 +2003,7 @@
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>（空表）</t>
+          <t>170</t>
         </is>
       </c>
     </row>
@@ -1989,7 +2026,7 @@
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>（空表）</t>
+          <t>发放对象</t>
         </is>
       </c>
     </row>
@@ -2012,7 +2049,7 @@
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>（空表）</t>
+          <t>客户编号</t>
         </is>
       </c>
     </row>
@@ -2035,7 +2072,7 @@
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>（空表）</t>
+          <t>WX-00000000000007507893</t>
         </is>
       </c>
     </row>
@@ -2097,10 +2134,8 @@
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr"/>
-      <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t>（空表）</t>
-        </is>
+      <c r="E2" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -2120,10 +2155,8 @@
           <t>是</t>
         </is>
       </c>
-      <c r="E3" s="1" t="inlineStr">
-        <is>
-          <t>（空表）</t>
-        </is>
+      <c r="E3" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -2145,7 +2178,7 @@
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>（空表）</t>
+          <t>单品优惠</t>
         </is>
       </c>
     </row>
@@ -2168,7 +2201,7 @@
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>（空表）</t>
+          <t>fixed_period</t>
         </is>
       </c>
     </row>
@@ -2187,7 +2220,7 @@
       <c r="D6" s="1" t="inlineStr"/>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>（空表）</t>
+          <t>2026-09-09 16:50:00</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2239,7 @@
       <c r="D7" s="1" t="inlineStr"/>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>（空表）</t>
+          <t>2026-09-12 16:50:00</t>
         </is>
       </c>
     </row>
@@ -2223,10 +2256,8 @@
       </c>
       <c r="C8" s="1" t="inlineStr"/>
       <c r="D8" s="1" t="inlineStr"/>
-      <c r="E8" s="1" t="inlineStr">
-        <is>
-          <t>（空表）</t>
-        </is>
+      <c r="E8" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -2246,10 +2277,8 @@
           <t>是</t>
         </is>
       </c>
-      <c r="E9" s="1" t="inlineStr">
-        <is>
-          <t>（空表）</t>
-        </is>
+      <c r="E9" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -2271,7 +2300,7 @@
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>（空表）</t>
+          <t>已结束</t>
         </is>
       </c>
     </row>
@@ -2771,7 +2800,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2926,7 +2955,88 @@
       <c r="D8" s="1" t="inlineStr"/>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>按核销明细</t>
+          <t>一致</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>theoretical_activity_benefit</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>NUMERIC</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr"/>
+      <c r="D9" s="1" t="inlineStr"/>
+      <c r="E9" s="1" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>theoretical_coupon_benefit</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>NUMERIC</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr"/>
+      <c r="D10" s="1" t="inlineStr"/>
+      <c r="E10" s="1" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>gift_qty_entitled</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t>NUMERIC</t>
+        </is>
+      </c>
+      <c r="C11" s="1" t="inlineStr"/>
+      <c r="D11" s="1" t="inlineStr"/>
+      <c r="E11" s="1" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>gift_qty_actual</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>NUMERIC</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="inlineStr"/>
+      <c r="D12" s="1" t="inlineStr"/>
+      <c r="E12" s="1" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>formula_ref</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="C13" s="1" t="inlineStr"/>
+      <c r="D13" s="1" t="inlineStr"/>
+      <c r="E13" s="1" t="inlineStr">
+        <is>
+          <t>activity_rule.reduce_amount</t>
         </is>
       </c>
     </row>
@@ -3217,7 +3327,7 @@
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>06377c7423cf4c8296bb32e5ad14fe2c</t>
+          <t>cb3feb58aa314484a6d7306ca0f033b2</t>
         </is>
       </c>
     </row>
@@ -3370,7 +3480,7 @@
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>2026-10-05T12:10:35</t>
+          <t>2026-10-06T11:28:04</t>
         </is>
       </c>
     </row>
@@ -3543,7 +3653,7 @@
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>/workspace/mvp/archives/27742ceaab44a7fc-sources.zip</t>
+          <t>/workspace/docs/samples/kuaima-verified-standard/满减/standard.xlsx</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3676,7 @@
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>27742ceaab44a7fc1cedeab440955abec5a12ee4bcb3b64a88fba776839123aa</t>
+          <t>sample-满减</t>
         </is>
       </c>
     </row>
@@ -3588,7 +3698,7 @@
         </is>
       </c>
       <c r="E7" s="1" t="n">
-        <v>5068081</v>
+        <v>5474150</v>
       </c>
     </row>
   </sheetData>
@@ -4878,7 +4988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4919,15 +5029,30 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>theoretical_activity_benefit</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>theoretical_coupon_benefit</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>consistent_orders</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>participating_orders</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>released_orders</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -4958,12 +5083,21 @@
         <v>200</v>
       </c>
       <c r="H2" s="1" t="n">
+        <v>2040</v>
+      </c>
+      <c r="I2" s="1" t="n">
+        <v>200</v>
+      </c>
+      <c r="J2" s="1" t="n">
         <v>136</v>
       </c>
-      <c r="I2" s="1" t="n">
+      <c r="K2" s="1" t="n">
+        <v>136</v>
+      </c>
+      <c r="L2" s="1" t="n">
         <v>133</v>
       </c>
-      <c r="J2" s="1" t="inlineStr">
+      <c r="M2" s="1" t="inlineStr">
         <is>
           <t>calculated</t>
         </is>
@@ -4994,12 +5128,21 @@
         <v>0</v>
       </c>
       <c r="H3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="1" t="n">
         <v>98</v>
       </c>
-      <c r="I3" s="1" t="n">
+      <c r="K3" s="1" t="n">
         <v>98</v>
       </c>
-      <c r="J3" s="1" t="inlineStr">
+      <c r="L3" s="1" t="n">
+        <v>98</v>
+      </c>
+      <c r="M3" s="1" t="inlineStr">
         <is>
           <t>calculated</t>
         </is>
@@ -5043,7 +5186,7 @@
         </is>
       </c>
       <c r="B2" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
@@ -5058,7 +5201,7 @@
         </is>
       </c>
       <c r="B3" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
@@ -5103,7 +5246,7 @@
         </is>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
@@ -5118,7 +5261,7 @@
         </is>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="C7" s="1" t="inlineStr">
         <is>
@@ -5152,7 +5295,7 @@
       </c>
       <c r="C9" s="1" t="inlineStr">
         <is>
-          <t>calculation_run_id / import_batch_id / calc_date / release_cutoff / activity_benefit / coupon_benefit / total_benefit / released_activity_benefit / released_coupon_benefit / participating_orders / released_orders / status</t>
+          <t>calculation_run_id / import_batch_id / calc_date / release_cutoff / activity_benefit / coupon_benefit / total_benefit / released_activity_benefit / released_coupon_benefit / theoretical_activity_benefit / theoretical_coupon_benefit / consistent_orders / participating_orders / released_orders / status</t>
         </is>
       </c>
     </row>
@@ -5163,7 +5306,7 @@
         </is>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C10" s="1" t="inlineStr">
         <is>
@@ -5178,7 +5321,7 @@
         </is>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C11" s="1" t="inlineStr">
         <is>
@@ -5208,7 +5351,7 @@
         </is>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C13" s="1" t="inlineStr">
         <is>
@@ -5223,7 +5366,7 @@
         </is>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C14" s="1" t="inlineStr">
         <is>
@@ -5272,7 +5415,7 @@
       </c>
       <c r="C17" s="1" t="inlineStr">
         <is>
-          <t>entitlement_check_id / calculation_run_id / order_id / activity_benefit / coupon_benefit / total_benefit / consistency</t>
+          <t>entitlement_check_id / calculation_run_id / order_id / activity_benefit / coupon_benefit / total_benefit / consistency / theoretical_activity_benefit / theoretical_coupon_benefit / gift_qty_entitled / gift_qty_actual / formula_ref</t>
         </is>
       </c>
     </row>
@@ -5561,7 +5704,11 @@
       </c>
       <c r="C7" s="1" t="inlineStr"/>
       <c r="D7" s="1" t="inlineStr"/>
-      <c r="E7" s="1" t="inlineStr"/>
+      <c r="E7" s="1" t="inlineStr">
+        <is>
+          <t>阶梯</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -5576,7 +5723,11 @@
       </c>
       <c r="C8" s="1" t="inlineStr"/>
       <c r="D8" s="1" t="inlineStr"/>
-      <c r="E8" s="1" t="inlineStr"/>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-31 10:58:00</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
@@ -5591,7 +5742,11 @@
       </c>
       <c r="C9" s="1" t="inlineStr"/>
       <c r="D9" s="1" t="inlineStr"/>
-      <c r="E9" s="1" t="inlineStr"/>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-17 23:59:00</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
@@ -5606,7 +5761,11 @@
       </c>
       <c r="C10" s="1" t="inlineStr"/>
       <c r="D10" s="1" t="inlineStr"/>
-      <c r="E10" s="1" t="inlineStr"/>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
@@ -5621,7 +5780,11 @@
       </c>
       <c r="C11" s="1" t="inlineStr"/>
       <c r="D11" s="1" t="inlineStr"/>
-      <c r="E11" s="1" t="inlineStr"/>
+      <c r="E11" s="1" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
@@ -5636,7 +5799,11 @@
       </c>
       <c r="C12" s="1" t="inlineStr"/>
       <c r="D12" s="1" t="inlineStr"/>
-      <c r="E12" s="1" t="inlineStr"/>
+      <c r="E12" s="1" t="inlineStr">
+        <is>
+          <t>已结束</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5696,10 +5863,8 @@
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr"/>
-      <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t>（空表）</t>
-        </is>
+      <c r="E2" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -5719,10 +5884,8 @@
           <t>是</t>
         </is>
       </c>
-      <c r="E3" s="1" t="inlineStr">
-        <is>
-          <t>（空表）</t>
-        </is>
+      <c r="E3" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -5744,7 +5907,7 @@
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>（空表）</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -5767,7 +5930,7 @@
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>（空表）</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -5790,7 +5953,7 @@
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>（空表）</t>
+          <t>立减</t>
         </is>
       </c>
     </row>
@@ -5807,11 +5970,7 @@
       </c>
       <c r="C7" s="1" t="inlineStr"/>
       <c r="D7" s="1" t="inlineStr"/>
-      <c r="E7" s="1" t="inlineStr">
-        <is>
-          <t>（空表）</t>
-        </is>
-      </c>
+      <c r="E7" s="1" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -5826,11 +5985,7 @@
       </c>
       <c r="C8" s="1" t="inlineStr"/>
       <c r="D8" s="1" t="inlineStr"/>
-      <c r="E8" s="1" t="inlineStr">
-        <is>
-          <t>（空表）</t>
-        </is>
-      </c>
+      <c r="E8" s="1" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
@@ -5845,10 +6000,8 @@
       </c>
       <c r="C9" s="1" t="inlineStr"/>
       <c r="D9" s="1" t="inlineStr"/>
-      <c r="E9" s="1" t="inlineStr">
-        <is>
-          <t>（空表）</t>
-        </is>
+      <c r="E9" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -5864,11 +6017,7 @@
       </c>
       <c r="C10" s="1" t="inlineStr"/>
       <c r="D10" s="1" t="inlineStr"/>
-      <c r="E10" s="1" t="inlineStr">
-        <is>
-          <t>（空表）</t>
-        </is>
-      </c>
+      <c r="E10" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6393,10 +6542,8 @@
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr"/>
-      <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t>（空表）</t>
-        </is>
+      <c r="E2" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -6416,10 +6563,8 @@
           <t>是</t>
         </is>
       </c>
-      <c r="E3" s="1" t="inlineStr">
-        <is>
-          <t>（空表）</t>
-        </is>
+      <c r="E3" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -6441,7 +6586,7 @@
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>（空表）</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -6464,7 +6609,7 @@
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>（空表）</t>
+          <t>金额</t>
         </is>
       </c>
     </row>
@@ -6481,10 +6626,8 @@
       </c>
       <c r="C6" s="1" t="inlineStr"/>
       <c r="D6" s="1" t="inlineStr"/>
-      <c r="E6" s="1" t="inlineStr">
-        <is>
-          <t>（空表）</t>
-        </is>
+      <c r="E6" s="1" t="n">
+        <v>300</v>
       </c>
     </row>
     <row r="7">
@@ -6500,10 +6643,8 @@
       </c>
       <c r="C7" s="1" t="inlineStr"/>
       <c r="D7" s="1" t="inlineStr"/>
-      <c r="E7" s="1" t="inlineStr">
-        <is>
-          <t>（空表）</t>
-        </is>
+      <c r="E7" s="1" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="8">
@@ -6519,10 +6660,8 @@
       </c>
       <c r="C8" s="1" t="inlineStr"/>
       <c r="D8" s="1" t="inlineStr"/>
-      <c r="E8" s="1" t="inlineStr">
-        <is>
-          <t>（空表）</t>
-        </is>
+      <c r="E8" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Import 羿柏 facts from the original MVP into ROI
The original library already has dealer 羿柏 / 舟谱 redemptions. Project them
into standard workbooks, import beside Kuaima, and compute ROI with the same
formula. Parse 1箱=24瓶 as 24 bottles, not the leading 1.

Co-authored-by: peggyzhan1 <peggyzhan1@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/samples/kuaima-verified-standard/ec101_standard库结构与当前数据.xlsx
+++ b/docs/samples/kuaima-verified-standard/ec101_standard库结构与当前数据.xlsx
@@ -2683,7 +2683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2786,6 +2786,72 @@
         </is>
       </c>
       <c r="G3" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>羿柏</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>舟谱</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>calculated</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>羿柏</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>舟谱</t>
+        </is>
+      </c>
+      <c r="D5" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="inlineStr">
+        <is>
+          <t>calculated</t>
+        </is>
+      </c>
+      <c r="G5" s="1" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3327,7 +3393,7 @@
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>cb3feb58aa314484a6d7306ca0f033b2</t>
+          <t>cc66938192404dbc80e321958245aa73</t>
         </is>
       </c>
     </row>
@@ -3480,7 +3546,7 @@
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>2026-10-06T11:28:04</t>
+          <t>2026-10-07T05:23:44</t>
         </is>
       </c>
     </row>
@@ -4988,7 +5054,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5143,6 +5209,96 @@
         <v>98</v>
       </c>
       <c r="M3" s="1" t="inlineStr">
+        <is>
+          <t>calculated</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>675</v>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="1" t="n">
+        <v>555</v>
+      </c>
+      <c r="G4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="1" t="n">
+        <v>45</v>
+      </c>
+      <c r="L4" s="1" t="n">
+        <v>37</v>
+      </c>
+      <c r="M4" s="1" t="inlineStr">
+        <is>
+          <t>calculated</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="1" t="n">
+        <v>142</v>
+      </c>
+      <c r="L5" s="1" t="n">
+        <v>142</v>
+      </c>
+      <c r="M5" s="1" t="inlineStr">
         <is>
           <t>calculated</t>
         </is>
@@ -5186,7 +5342,7 @@
         </is>
       </c>
       <c r="B2" s="1" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
@@ -5201,7 +5357,7 @@
         </is>
       </c>
       <c r="B3" s="1" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
@@ -5216,7 +5372,7 @@
         </is>
       </c>
       <c r="B4" s="1" t="n">
-        <v>234</v>
+        <v>421</v>
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
@@ -5231,7 +5387,7 @@
         </is>
       </c>
       <c r="B5" s="1" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
@@ -5246,7 +5402,7 @@
         </is>
       </c>
       <c r="B6" s="1" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
@@ -5261,7 +5417,7 @@
         </is>
       </c>
       <c r="B7" s="1" t="n">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="C7" s="1" t="inlineStr">
         <is>
@@ -5276,7 +5432,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>3</v>
+        <v>198</v>
       </c>
       <c r="C8" s="1" t="inlineStr">
         <is>
@@ -5291,7 +5447,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C9" s="1" t="inlineStr">
         <is>
@@ -5381,7 +5537,7 @@
         </is>
       </c>
       <c r="B15" s="1" t="n">
-        <v>4584</v>
+        <v>4764</v>
       </c>
       <c r="C15" s="1" t="inlineStr">
         <is>
@@ -5396,7 +5552,7 @@
         </is>
       </c>
       <c r="B16" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C16" s="1" t="inlineStr">
         <is>
@@ -5411,7 +5567,7 @@
         </is>
       </c>
       <c r="B17" s="1" t="n">
-        <v>234</v>
+        <v>421</v>
       </c>
       <c r="C17" s="1" t="inlineStr">
         <is>
@@ -5426,7 +5582,7 @@
         </is>
       </c>
       <c r="B18" s="1" t="n">
-        <v>3021</v>
+        <v>3205</v>
       </c>
       <c r="C18" s="1" t="inlineStr">
         <is>
@@ -5441,7 +5597,7 @@
         </is>
       </c>
       <c r="B19" s="1" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C19" s="1" t="inlineStr">
         <is>
@@ -5456,7 +5612,7 @@
         </is>
       </c>
       <c r="B20" s="1" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C20" s="1" t="inlineStr">
         <is>
@@ -5486,7 +5642,7 @@
         </is>
       </c>
       <c r="B22" s="1" t="n">
-        <v>3021</v>
+        <v>3208</v>
       </c>
       <c r="C22" s="1" t="inlineStr">
         <is>
@@ -5501,7 +5657,7 @@
         </is>
       </c>
       <c r="B23" s="1" t="n">
-        <v>62411</v>
+        <v>66575</v>
       </c>
       <c r="C23" s="1" t="inlineStr">
         <is>
@@ -5516,7 +5672,7 @@
         </is>
       </c>
       <c r="B24" s="1" t="n">
-        <v>18347</v>
+        <v>19440</v>
       </c>
       <c r="C24" s="1" t="inlineStr">
         <is>
@@ -5531,7 +5687,7 @@
         </is>
       </c>
       <c r="B25" s="1" t="n">
-        <v>234</v>
+        <v>421</v>
       </c>
       <c r="C25" s="1" t="inlineStr">
         <is>

</xml_diff>